<commit_message>
feat: Agregar funcionalidad de consulta de notas en tiempo real.
</commit_message>
<xml_diff>
--- a/plantilla-BD/ChatBot.xlsx
+++ b/plantilla-BD/ChatBot.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="66">
   <si>
     <t>id_tutor</t>
   </si>
@@ -32,7 +32,7 @@
     <t>estado_tutor</t>
   </si>
   <si>
-    <t>Juan</t>
+    <t>Rosalía</t>
   </si>
   <si>
     <t>Matemática</t>
@@ -53,7 +53,7 @@
     <t>Literatura</t>
   </si>
   <si>
-    <t>José</t>
+    <t>Cleopatra</t>
   </si>
   <si>
     <t>Historia</t>
@@ -92,7 +92,7 @@
     <t>09:00</t>
   </si>
   <si>
-    <t>Ocupado</t>
+    <t>Libre</t>
   </si>
   <si>
     <t>2</t>
@@ -107,6 +107,9 @@
     <t>10:00</t>
   </si>
   <si>
+    <t>Ocupado</t>
+  </si>
+  <si>
     <t>3</t>
   </si>
   <si>
@@ -117,9 +120,6 @@
   </si>
   <si>
     <t>11:00</t>
-  </si>
-  <si>
-    <t>Libre</t>
   </si>
   <si>
     <t>4</t>
@@ -179,10 +179,10 @@
     <t>estado</t>
   </si>
   <si>
-    <t>Cancelado</t>
+    <t>Agendada</t>
   </si>
   <si>
-    <t>Agendada</t>
+    <t>Finalizada</t>
   </si>
   <si>
     <t>telegram_user</t>
@@ -197,7 +197,7 @@
     <t>datos_parciales</t>
   </si>
   <si>
-    <t>cancelando_tutoria</t>
+    <t>esperando_menu</t>
   </si>
   <si>
     <t>{}</t>
@@ -209,7 +209,10 @@
     <t>nombre_completo</t>
   </si>
   <si>
-    <t>Ricardo Jom</t>
+    <t>puntos</t>
+  </si>
+  <si>
+    <t>Marco Raquec</t>
   </si>
 </sst>
 </file>
@@ -261,13 +264,27 @@
       <patternFill patternType="lightGray"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="29">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -326,17 +343,32 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -457,7 +489,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E6" displayName="Tabla_1" name="Tabla_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E21" displayName="Tabla_1" name="Tabla_1" id="1">
   <tableColumns count="5">
     <tableColumn name="id_tutor" id="1"/>
     <tableColumn name="id_telegram" id="2"/>
@@ -511,10 +543,11 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:B25" displayName="Tabla_5" name="Tabla_5" id="5">
-  <tableColumns count="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:C25" displayName="Tabla_5" name="Tabla_5" id="5">
+  <tableColumns count="3">
     <tableColumn name="id_usuario" id="1"/>
     <tableColumn name="nombre_completo" id="2"/>
+    <tableColumn name="puntos" id="3"/>
   </tableColumns>
   <tableStyleInfo name="estudiantes-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
@@ -875,12 +908,12 @@
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
     </row>
-    <row r="7">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
+    <row r="7" ht="22.5" customHeight="1">
+      <c r="A7" s="3"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
@@ -890,12 +923,12 @@
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
     </row>
-    <row r="8">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
+    <row r="8" ht="22.5" customHeight="1">
+      <c r="A8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
@@ -905,12 +938,12 @@
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
     </row>
-    <row r="9">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
+    <row r="9" ht="22.5" customHeight="1">
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
@@ -920,12 +953,12 @@
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
     </row>
-    <row r="10">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
+    <row r="10" ht="22.5" customHeight="1">
+      <c r="A10" s="3"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
@@ -935,12 +968,12 @@
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
     </row>
-    <row r="11">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
+    <row r="11" ht="22.5" customHeight="1">
+      <c r="A11" s="3"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
@@ -950,12 +983,12 @@
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
     </row>
-    <row r="12">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
+    <row r="12" ht="22.5" customHeight="1">
+      <c r="A12" s="3"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
@@ -965,12 +998,12 @@
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
     </row>
-    <row r="13">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
+    <row r="13" ht="22.5" customHeight="1">
+      <c r="A13" s="3"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
@@ -980,12 +1013,12 @@
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
     </row>
-    <row r="14">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
+    <row r="14" ht="22.5" customHeight="1">
+      <c r="A14" s="3"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
@@ -995,12 +1028,12 @@
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
     </row>
-    <row r="15">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
+    <row r="15" ht="22.5" customHeight="1">
+      <c r="A15" s="3"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
@@ -1010,12 +1043,12 @@
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
     </row>
-    <row r="16">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
+    <row r="16" ht="22.5" customHeight="1">
+      <c r="A16" s="3"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
@@ -1025,12 +1058,12 @@
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
     </row>
-    <row r="17">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
+    <row r="17" ht="22.5" customHeight="1">
+      <c r="A17" s="3"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
@@ -1040,12 +1073,12 @@
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
     </row>
-    <row r="18">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
+    <row r="18" ht="22.5" customHeight="1">
+      <c r="A18" s="3"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
@@ -1055,12 +1088,12 @@
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
     </row>
-    <row r="19">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
+    <row r="19" ht="22.5" customHeight="1">
+      <c r="A19" s="3"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
@@ -1070,12 +1103,12 @@
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
     </row>
-    <row r="20">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
+    <row r="20" ht="22.5" customHeight="1">
+      <c r="A20" s="3"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
@@ -1085,12 +1118,12 @@
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
     </row>
-    <row r="21">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
+    <row r="21" ht="22.5" customHeight="1">
+      <c r="A21" s="3"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -4169,7 +4202,7 @@
     </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="A2:A6">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="A2:A21">
       <formula1>AND(ISNUMBER(A2),(NOT(OR(NOT(ISERROR(DATEVALUE(A2))), AND(ISNUMBER(A2), LEFT(CELL("format", A2))="D")))))</formula1>
     </dataValidation>
   </dataValidations>
@@ -4189,6 +4222,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="18.13"/>
     <col customWidth="1" min="2" max="2" width="14.5"/>
+    <col customWidth="1" min="3" max="3" width="18.25"/>
     <col customWidth="1" min="4" max="4" width="16.0"/>
     <col customWidth="1" min="5" max="5" width="14.75"/>
     <col customWidth="1" min="6" max="6" width="15.75"/>
@@ -4267,7 +4301,7 @@
         <v>29</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -4280,22 +4314,22 @@
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
@@ -4323,7 +4357,7 @@
         <v>37</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
@@ -4345,13 +4379,13 @@
         <v>39</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>40</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
@@ -4379,7 +4413,7 @@
         <v>43</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
@@ -4407,7 +4441,7 @@
         <v>47</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
@@ -4588,7 +4622,6 @@
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
@@ -13540,22 +13573,22 @@
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="11">
-        <v>1.783947590731E12</v>
+        <v>1.784214500614E12</v>
       </c>
       <c r="B2" s="12">
-        <v>8.471796813E9</v>
+        <v>7.511039778E9</v>
       </c>
       <c r="C2" s="11">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E2" s="13">
-        <v>46216.0</v>
+        <v>46260.0</v>
       </c>
       <c r="F2" s="14">
-        <v>0.2916666666666667</v>
+        <v>0.375</v>
       </c>
       <c r="G2" s="11" t="s">
         <v>54</v>
@@ -13570,10 +13603,10 @@
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="4">
-        <v>1.783947390196E12</v>
+        <v>1.78429543376E12</v>
       </c>
       <c r="B3" s="12">
-        <v>8.471796813E9</v>
+        <v>7.511039778E9</v>
       </c>
       <c r="C3" s="11">
         <v>2.0</v>
@@ -13582,7 +13615,7 @@
         <v>6</v>
       </c>
       <c r="E3" s="13">
-        <v>46217.0</v>
+        <v>46288.0</v>
       </c>
       <c r="F3" s="14">
         <v>0.3333333333333333</v>
@@ -13600,25 +13633,25 @@
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="15">
-        <v>1.783947590731E12</v>
+        <v>1.784214500614E12</v>
       </c>
       <c r="B4" s="15">
-        <v>8.471796813E9</v>
+        <v>7.511039778E9</v>
       </c>
       <c r="C4" s="4">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E4" s="16">
-        <v>46216.0</v>
+        <v>46260.0</v>
       </c>
       <c r="F4" s="17">
-        <v>0.2916666666666667</v>
+        <v>0.375</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
@@ -13629,13 +13662,27 @@
       <c r="N4" s="2"/>
     </row>
     <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="4"/>
+      <c r="A5" s="15">
+        <v>1.784291303746E12</v>
+      </c>
+      <c r="B5" s="15">
+        <v>7.511039778E9</v>
+      </c>
+      <c r="C5" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="16">
+        <v>46163.0</v>
+      </c>
+      <c r="F5" s="17">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>54</v>
+      </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -13645,13 +13692,27 @@
       <c r="N5" s="2"/>
     </row>
     <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="15"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="16"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="4"/>
+      <c r="A6" s="15">
+        <v>1.78429543376E12</v>
+      </c>
+      <c r="B6" s="15">
+        <v>7.511039778E9</v>
+      </c>
+      <c r="C6" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="16">
+        <v>46288.0</v>
+      </c>
+      <c r="F6" s="17">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>55</v>
+      </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
@@ -13693,12 +13754,12 @@
       <c r="N8" s="2"/>
     </row>
     <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="18"/>
+      <c r="A9" s="15"/>
       <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
+      <c r="C9" s="4"/>
       <c r="D9" s="4"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="17"/>
       <c r="G9" s="4"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -13709,12 +13770,12 @@
       <c r="N9" s="2"/>
     </row>
     <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="18"/>
+      <c r="A10" s="15"/>
       <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
+      <c r="C10" s="4"/>
       <c r="D10" s="4"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="17"/>
       <c r="G10" s="4"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
@@ -16801,7 +16862,7 @@
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="20">
-        <v>8.471796813E9</v>
+        <v>7.511039778E9</v>
       </c>
       <c r="B2" s="21" t="s">
         <v>60</v>
@@ -16812,6 +16873,12 @@
       <c r="D2" s="21" t="s">
         <v>61</v>
       </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="22"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -16828,7 +16895,9 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
+    <col customWidth="1" min="1" max="1" width="14.88"/>
     <col customWidth="1" min="2" max="2" width="36.0"/>
+    <col customWidth="1" min="3" max="3" width="18.0"/>
     <col customWidth="1" min="5" max="5" width="16.63"/>
   </cols>
   <sheetData>
@@ -16839,9 +16908,11 @@
       <c r="B1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
+      <c r="C1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
@@ -16855,13 +16926,15 @@
       <c r="P1" s="2"/>
     </row>
     <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="23">
-        <v>8.471796813E9</v>
+      <c r="A2" s="25">
+        <v>7.511039778E9</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
-      <c r="C2" s="8"/>
+      <c r="C2" s="26">
+        <v>20.0</v>
+      </c>
       <c r="D2" s="8"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
@@ -16877,9 +16950,9 @@
       <c r="P2" s="2"/>
     </row>
     <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="18"/>
-      <c r="B3" s="18"/>
-      <c r="C3" s="2"/>
+      <c r="A3" s="15"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="27"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
@@ -16895,9 +16968,9 @@
       <c r="P3" s="2"/>
     </row>
     <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="18"/>
-      <c r="B4" s="18"/>
-      <c r="C4" s="2"/>
+      <c r="A4" s="15"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="27"/>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
@@ -16915,7 +16988,7 @@
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="18"/>
       <c r="B5" s="18"/>
-      <c r="C5" s="2"/>
+      <c r="C5" s="28"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
@@ -16933,7 +17006,7 @@
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="18"/>
       <c r="B6" s="18"/>
-      <c r="C6" s="2"/>
+      <c r="C6" s="28"/>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
@@ -16951,7 +17024,7 @@
     <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="18"/>
       <c r="B7" s="18"/>
-      <c r="C7" s="2"/>
+      <c r="C7" s="28"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
@@ -16969,7 +17042,7 @@
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="18"/>
       <c r="B8" s="18"/>
-      <c r="C8" s="2"/>
+      <c r="C8" s="28"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
@@ -16987,7 +17060,7 @@
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="18"/>
       <c r="B9" s="18"/>
-      <c r="C9" s="2"/>
+      <c r="C9" s="28"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
@@ -17005,7 +17078,7 @@
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="18"/>
       <c r="B10" s="18"/>
-      <c r="C10" s="2"/>
+      <c r="C10" s="28"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -17023,7 +17096,7 @@
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="18"/>
       <c r="B11" s="18"/>
-      <c r="C11" s="2"/>
+      <c r="C11" s="28"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
@@ -17041,7 +17114,7 @@
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="18"/>
       <c r="B12" s="18"/>
-      <c r="C12" s="2"/>
+      <c r="C12" s="28"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
@@ -17059,7 +17132,7 @@
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="18"/>
       <c r="B13" s="18"/>
-      <c r="C13" s="2"/>
+      <c r="C13" s="28"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
@@ -17077,7 +17150,7 @@
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="18"/>
       <c r="B14" s="18"/>
-      <c r="C14" s="2"/>
+      <c r="C14" s="28"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
@@ -17095,7 +17168,7 @@
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="18"/>
       <c r="B15" s="18"/>
-      <c r="C15" s="2"/>
+      <c r="C15" s="28"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
@@ -17113,7 +17186,7 @@
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="18"/>
       <c r="B16" s="18"/>
-      <c r="C16" s="2"/>
+      <c r="C16" s="28"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
@@ -17131,7 +17204,7 @@
     <row r="17" ht="22.5" customHeight="1">
       <c r="A17" s="18"/>
       <c r="B17" s="18"/>
-      <c r="C17" s="2"/>
+      <c r="C17" s="28"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
@@ -17149,7 +17222,7 @@
     <row r="18" ht="22.5" customHeight="1">
       <c r="A18" s="18"/>
       <c r="B18" s="18"/>
-      <c r="C18" s="2"/>
+      <c r="C18" s="28"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
@@ -17167,7 +17240,7 @@
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="18"/>
       <c r="B19" s="18"/>
-      <c r="C19" s="2"/>
+      <c r="C19" s="28"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
@@ -17185,7 +17258,7 @@
     <row r="20" ht="22.5" customHeight="1">
       <c r="A20" s="18"/>
       <c r="B20" s="18"/>
-      <c r="C20" s="2"/>
+      <c r="C20" s="28"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
@@ -17203,7 +17276,7 @@
     <row r="21" ht="22.5" customHeight="1">
       <c r="A21" s="18"/>
       <c r="B21" s="18"/>
-      <c r="C21" s="2"/>
+      <c r="C21" s="28"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
@@ -17221,7 +17294,7 @@
     <row r="22" ht="22.5" customHeight="1">
       <c r="A22" s="18"/>
       <c r="B22" s="18"/>
-      <c r="C22" s="2"/>
+      <c r="C22" s="28"/>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
@@ -17239,7 +17312,7 @@
     <row r="23" ht="22.5" customHeight="1">
       <c r="A23" s="18"/>
       <c r="B23" s="18"/>
-      <c r="C23" s="2"/>
+      <c r="C23" s="28"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
@@ -17257,7 +17330,7 @@
     <row r="24" ht="22.5" customHeight="1">
       <c r="A24" s="18"/>
       <c r="B24" s="18"/>
-      <c r="C24" s="2"/>
+      <c r="C24" s="28"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
@@ -17275,7 +17348,7 @@
     <row r="25" ht="22.5" customHeight="1">
       <c r="A25" s="18"/>
       <c r="B25" s="18"/>
-      <c r="C25" s="2"/>
+      <c r="C25" s="28"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>

</xml_diff>